<commit_message>
feat(resources): 2단계 — 자원 관리 재편
백엔드:
- 계약 생성에 용도↔직무↔형태 교차 검증 (클린차량↔클리너↔직영·협력 필수,
  배송용↔라이더↔engagement 금지) — 400 VALIDATION_FAILED
- rider_bike_contracts.engagement_type 노출 (V57) + 매칭 엑셀 이원화
  (배송: 구독/렌탈+인수/반납, 클리닝: 직영/협력+CUSTOM 템플릿)
- 등급 미판정 되돌리기 clearSkillLevel 플래그 (JSON null 무변경 문제 회피)
- 차량 운영상태 이력 bikeId 필터 조회

프론트:
- 자원 관리 페이지 서버 fetch → props 단일 소스, 갱신은 router.refresh()
- 차량 상세: 함체 체크(배송용만, 장비 도메인 재사용), 매칭 요약,
  운영상태 이력 — 관제 floating 패널과 동일 다이얼로그 재사용 (returnTo)
- 이용자 상세: 기본/직무/팀/등급(초보·고수·미판정)/보험 수정 + 교육 기록
- 단건 등록 다이얼로그 3종 (차량·이용자·매칭 — 용도별 폼 분기)
- 표 검색 input, 매칭 표 직영/협력 표시, skillLevel 타입 V58 정합
- 죽은 overview create/delete 액션·DeleteVehicleButton 제거

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/development/backend/src/main/resources/templates/excel/matching-template.xlsx
+++ b/development/backend/src/main/resources/templates/excel/matching-template.xlsx
@@ -631,14 +631,14 @@
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>계약형태 *
-(구독/렌탈)</t>
+          <t>계약형태
+(구독/렌탈 — 배송 전용)</t>
         </is>
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>인수방식 *
-(인수형/반납형)</t>
+          <t>계약 형태 *
+(배송: 인수형/반납형 · 클리닝: 직영/협력)</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">

</xml_diff>